<commit_message>
Renska opp i språk og div
</commit_message>
<xml_diff>
--- a/data/appliances.xlsx
+++ b/data/appliances.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stuja\OneDrive\Dokumenter\Studie\0. Etterstudium\Eninf Oblig 1\git2\in5410_intelligent_load_scheduling\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{877DB33F-98D4-4D76-A591-07231DE4B6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D445FE0C-D14F-4597-B577-908A9B444946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>navn</t>
   </si>
@@ -36,12 +36,6 @@
     <t>d</t>
   </si>
   <si>
-    <t>vindu_start</t>
-  </si>
-  <si>
-    <t>vindu_slutt</t>
-  </si>
-  <si>
     <t>kan_pauses</t>
   </si>
   <si>
@@ -64,6 +58,18 @@
   </si>
   <si>
     <t>3.0</t>
+  </si>
+  <si>
+    <t>vindu</t>
+  </si>
+  <si>
+    <t>65-81, 117-139</t>
+  </si>
+  <si>
+    <t>65-121</t>
+  </si>
+  <si>
+    <t>37-132</t>
   </si>
 </sst>
 </file>
@@ -421,10 +427,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="34.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -435,84 +441,72 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="C2" s="3">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="3">
-        <v>2</v>
-      </c>
-      <c r="D2" s="3">
+      <c r="C3" s="3">
         <v>16</v>
       </c>
-      <c r="E2" s="3">
-        <v>24</v>
-      </c>
-      <c r="F2" s="3">
-        <v>0</v>
-      </c>
-      <c r="G2" s="4">
-        <v>0</v>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3">
-        <v>4</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0</v>
-      </c>
-      <c r="E3" s="3">
-        <v>24</v>
-      </c>
-      <c r="F3" s="3">
+      <c r="C4" s="3">
+        <v>20</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3">
         <v>1</v>
       </c>
-      <c r="G3" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3">
-        <v>5</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0</v>
-      </c>
-      <c r="E4" s="3">
-        <v>10</v>
-      </c>
-      <c r="F4" s="3">
-        <v>1</v>
-      </c>
-      <c r="G4" s="4">
+      <c r="F4" s="4">
         <v>0</v>
       </c>
     </row>

</xml_diff>